<commit_message>
Rebuild RA_Moose_Scorpion and RA_GECKO per same EHS revalidation feedback
Applies the same fix used on RA_InfurrowElk.xlsx: tasks broken into
real physical steps (20 rows each, was 10/12), controls describe
administrative + engineering + LOTO explicitly, EPP declared on every
row (cleanroom gear), Arranque and Emergencia sections added, and
nivelControl chosen to match the actual control described.

The "documento" field now carries only the bare visual-aid (AV)
document numbers per the user's instruction, cross-referenced from the
AV folder screenshot they sent (16-AT40-3318-000XX series) -- all 8
GECKO numbers confirmed, 7 of 8 Moose/Scorpion confirmed (Front Assy
Moose's number was cropped/illegible, left as pending).
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/RA_GECKO.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/RA_GECKO.xlsx
@@ -6395,7 +6395,7 @@
     <row r="2" spans="1:19" s="20" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Estaciones GECKO de Atornillado Automático (VSS1H-6050-001 a 006, MS-550-001, MS-550-002)</t>
+          <t xml:space="preserve">REVALIDACION: Estaciones GECKO de Atornillado Automático (VSS1H-6050-001 a 006, MS-550-001, MS-550-002)</t>
         </is>
       </c>
       <c r="B2" s="127"/>
@@ -6435,7 +6435,7 @@
       <c r="C3" s="127"/>
       <c r="D3" s="52" t="inlineStr">
         <is>
-          <t xml:space="preserve">18/09/2026</t>
+          <t xml:space="preserve">30/09/2026</t>
         </is>
       </c>
       <c r="E3" s="143" t="s">
@@ -6606,12 +6606,12 @@
       </c>
       <c r="B8" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - carga de pieza con robot gantry en posición de reposo</t>
+          <t xml:space="preserve">Carga de pieza en la fixtura y clampeo manual</t>
         </is>
       </c>
       <c r="C8" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El operador coloca la pieza manualmente en la fixtura, la clampea con los 2 clamps y sale del área antes de dar avance</t>
+          <t xml:space="preserve">Paso 1 de 2: el operador coloca la pieza manualmente en la fixtura, en posición de reposo del gantry</t>
         </is>
       </c>
       <c r="D8" s="56" t="inlineStr">
@@ -6655,12 +6655,19 @@
       </c>
       <c r="L8" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; el control es por cortinas de seguridad en el área central.</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M8" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Estaciones GECKO</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N8" s="57" t="inlineStr">
@@ -6692,42 +6699,42 @@
       </c>
       <c r="B9" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - movimiento del slider en X (y eje adicional en algunas estaciones)</t>
+          <t xml:space="preserve">Carga de pieza en la fixtura y clampeo manual</t>
         </is>
       </c>
       <c r="C9" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El slider mueve la fixtura con la pieza clampeada hacia la posición de atornillado durante el ciclo automático</t>
+          <t xml:space="preserve">Paso 2 de 2: cierra los 2 clamps manuales de la fixtura y sale del área antes de dar avance</t>
         </is>
       </c>
       <c r="D9" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mecanico</t>
+          <t xml:space="preserve">Ergonomía</t>
         </is>
       </c>
       <c r="E9" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Partes móviles</t>
+          <t xml:space="preserve">Movimientos repetitivos</t>
         </is>
       </c>
       <c r="F9" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laceración</t>
+          <t xml:space="preserve">Fatiga muscular</t>
         </is>
       </c>
       <c r="G9" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control</t>
+          <t xml:space="preserve">Influencia</t>
         </is>
       </c>
       <c r="H9" s="57" t="inlineStr">
         <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="I9" s="57" t="inlineStr">
+        <is>
           <t xml:space="preserve">3</t>
-        </is>
-      </c>
-      <c r="I9" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="J9" s="51">
@@ -6736,17 +6743,24 @@
       </c>
       <c r="K9" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensores</t>
+          <t xml:space="preserve">ergonomía</t>
         </is>
       </c>
       <c r="L9" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; el control es por cortinas de seguridad en el área central.</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M9" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Estaciones GECKO</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N9" s="57" t="inlineStr">
@@ -6756,7 +6770,7 @@
       </c>
       <c r="O9" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="P9" s="61">
@@ -6778,12 +6792,12 @@
       </c>
       <c r="B10" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - movimiento/rotación del cabezal de torque</t>
+          <t xml:space="preserve">Verificación Poka Yoke de presencia/orientación de la pieza</t>
         </is>
       </c>
       <c r="C10" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El cabezal de torque se mueve a la posición del feeder, recoge el tornillo y se mueve a la posición de atornillado</t>
+          <t xml:space="preserve">El sensor/pin Poka Yoke de la fixtura verifica que la pieza esté correctamente orientada antes de permitir el ciclo; el operador puede tener contacto accidental con el mecanismo al cargar la pieza</t>
         </is>
       </c>
       <c r="D10" s="56" t="inlineStr">
@@ -6798,7 +6812,7 @@
       </c>
       <c r="F10" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fractura</t>
+          <t xml:space="preserve">Laceración</t>
         </is>
       </c>
       <c r="G10" s="56" t="inlineStr">
@@ -6808,12 +6822,12 @@
       </c>
       <c r="H10" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="I10" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J10" s="51">
@@ -6822,17 +6836,24 @@
       </c>
       <c r="K10" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensores</t>
+          <t xml:space="preserve">Resguardos mecánicos</t>
         </is>
       </c>
       <c r="L10" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; el control es por cortinas de seguridad en el área central (mismo set que protege gantry y slider).</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M10" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Estaciones GECKO</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N10" s="57" t="inlineStr">
@@ -6859,17 +6880,17 @@
     <row r="11" spans="1:19" s="19" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">No rutinario</t>
+          <t xml:space="preserve">Rutinario</t>
         </is>
       </c>
       <c r="B11" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mantenimiento - cambio de motor, eje o cable</t>
+          <t xml:space="preserve">Lectura de código con escáner fijo</t>
         </is>
       </c>
       <c r="C11" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El personal de mantenimiento cambia el switch de llave a modo mantenimiento y bloquea el switch general de energía antes de intervenir</t>
+          <t xml:space="preserve">El escáner fijo lee el código de la pieza/etiqueta antes o durante el ciclo; el operador puede golpearse con el escáner o golpear material al cargar/descargar</t>
         </is>
       </c>
       <c r="D11" s="56" t="inlineStr">
@@ -6884,7 +6905,7 @@
       </c>
       <c r="F11" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Atrapamiento</t>
+          <t xml:space="preserve">Laceración</t>
         </is>
       </c>
       <c r="G11" s="56" t="inlineStr">
@@ -6894,12 +6915,12 @@
       </c>
       <c r="H11" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="I11" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="J11" s="51">
@@ -6908,17 +6929,24 @@
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOTO</t>
+          <t xml:space="preserve">Resguardos mecánicos</t>
         </is>
       </c>
       <c r="L11" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; candado y tarjeta de bloqueo en el switch general.</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M11" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procedimiento LOTO de la estación</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N11" s="57" t="inlineStr">
@@ -6950,12 +6978,12 @@
       </c>
       <c r="B12" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - recolección de tornillo por succión de vacío en el feeder</t>
+          <t xml:space="preserve">Contacto con partes fijas de la fixtura (bordes/topes)</t>
         </is>
       </c>
       <c r="C12" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">La electroválvula de vacío recoge el tornillo del feeder antes de llevarlo a la posición de atornillado</t>
+          <t xml:space="preserve">El operador puede golpearse o atraparse los dedos con los bordes/topes fijos de la fixtura al colocar o retirar la pieza</t>
         </is>
       </c>
       <c r="D12" s="56" t="inlineStr">
@@ -6980,7 +7008,7 @@
       </c>
       <c r="H12" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="I12" s="57" t="inlineStr">
@@ -6999,12 +7027,19 @@
       </c>
       <c r="L12" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; guarda fija en el punto de recolección del feeder.</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M12" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Estaciones GECKO</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N12" s="57" t="inlineStr">
@@ -7031,32 +7066,32 @@
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">No rutinario</t>
+          <t xml:space="preserve">Rutinario</t>
         </is>
       </c>
       <c r="B13" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mantenimiento correctivo / solución de problemas eléctricos</t>
+          <t xml:space="preserve">Ciclo automático de atornillado (gantry, slider, cabezal de torque)</t>
         </is>
       </c>
       <c r="C13" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El personal de mantenimiento abre el gabinete/panel eléctrico de la estación para diagnóstico o reparación</t>
+          <t xml:space="preserve">Paso 1 de 3: el slider mueve la fixtura con la pieza clampeada hacia la posición de atornillado durante el ciclo automático; las cortinas de seguridad del área central impiden el acceso durante este movimiento</t>
         </is>
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eléctrico</t>
+          <t xml:space="preserve">Mecanico</t>
         </is>
       </c>
       <c r="E13" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conductores energizados</t>
+          <t xml:space="preserve">Partes móviles</t>
         </is>
       </c>
       <c r="F13" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrocución</t>
+          <t xml:space="preserve">Laceración</t>
         </is>
       </c>
       <c r="G13" s="56" t="inlineStr">
@@ -7066,7 +7101,7 @@
       </c>
       <c r="H13" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="I13" s="57" t="inlineStr">
@@ -7080,17 +7115,24 @@
       </c>
       <c r="K13" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOTO</t>
+          <t xml:space="preserve">sensores</t>
         </is>
       </c>
       <c r="L13" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guantes dieléctricos (clase según voltaje) y calzado aislante.</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M13" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procedimiento LOTO de la estación</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N13" s="57" t="inlineStr">
@@ -7100,7 +7142,7 @@
       </c>
       <c r="O13" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="P13" s="61">
@@ -7122,42 +7164,42 @@
       </c>
       <c r="B14" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manejo de materiales - clampeo manual de la pieza</t>
+          <t xml:space="preserve">Ciclo automático de atornillado (gantry, slider, cabezal de torque)</t>
         </is>
       </c>
       <c r="C14" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El operador coloca la pieza en la fixtura y cierra los 2 clamps manuales cada ciclo</t>
+          <t xml:space="preserve">Paso 2 de 3: el cabezal de torque se mueve a la posición del feeder, recoge el tornillo por succión de vacío y se mueve a la posición de atornillado</t>
         </is>
       </c>
       <c r="D14" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ergonomía</t>
+          <t xml:space="preserve">Mecanico</t>
         </is>
       </c>
       <c r="E14" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Movimientos repetitivos</t>
+          <t xml:space="preserve">Partes móviles</t>
         </is>
       </c>
       <c r="F14" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fatiga muscular</t>
+          <t xml:space="preserve">Fractura</t>
         </is>
       </c>
       <c r="G14" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Influencia</t>
+          <t xml:space="preserve">Control</t>
         </is>
       </c>
       <c r="H14" s="57" t="inlineStr">
         <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="I14" s="57" t="inlineStr">
+        <is>
           <t xml:space="preserve">2</t>
-        </is>
-      </c>
-      <c r="I14" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="J14" s="51">
@@ -7166,17 +7208,24 @@
       </c>
       <c r="K14" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">ergonomía</t>
+          <t xml:space="preserve">sensores</t>
         </is>
       </c>
       <c r="L14" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional.</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M14" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evaluación ergonómica de la estación</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N14" s="57" t="inlineStr">
@@ -7186,7 +7235,7 @@
       </c>
       <c r="O14" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="P14" s="61">
@@ -7203,17 +7252,17 @@
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">No rutinario</t>
+          <t xml:space="preserve">Rutinario</t>
         </is>
       </c>
       <c r="B15" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mantenimiento - energía neumática residual del sistema de vacío</t>
+          <t xml:space="preserve">Ciclo automático de atornillado (gantry, slider, cabezal de torque)</t>
         </is>
       </c>
       <c r="C15" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El personal de mantenimiento interviene la línea neumática de la electroválvula de vacío; actualmente no existe válvula de despresurización/bloqueo LOTO neumático (en proceso de compra)</t>
+          <t xml:space="preserve">Paso 3 de 3: el slider regresa la pieza a la posición frontal para que el operador la descargue</t>
         </is>
       </c>
       <c r="D15" s="56" t="inlineStr">
@@ -7223,22 +7272,22 @@
       </c>
       <c r="E15" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema de presión</t>
+          <t xml:space="preserve">Partes móviles</t>
         </is>
       </c>
       <c r="F15" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laceraciones</t>
+          <t xml:space="preserve">Laceración</t>
         </is>
       </c>
       <c r="G15" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Influencia</t>
+          <t xml:space="preserve">Control</t>
         </is>
       </c>
       <c r="H15" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="I15" s="57" t="inlineStr">
@@ -7252,17 +7301,24 @@
       </c>
       <c r="K15" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">inspecciones periódicas</t>
+          <t xml:space="preserve">Resguardos mecánicos</t>
         </is>
       </c>
       <c r="L15" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional. Riesgo bajo: solo succión de baja presión, sin pistones. Pendiente instalar válvula de despresurización/bloqueo LOTO neumático (en compra); mientras tanto solo se cuenta con inspección periódica del circuito.</t>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
         </is>
       </c>
       <c r="M15" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procedimiento LOTO de la estación (pendiente actualizar con válvula neumática)</t>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
         </is>
       </c>
       <c r="N15" s="57" t="inlineStr">
@@ -7272,7 +7328,7 @@
       </c>
       <c r="O15" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="P15" s="61">
@@ -7287,24 +7343,87 @@
       <c r="S15" s="57"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A16" s="55"/>
-      <c r="B16" s="55"/>
-      <c r="C16" s="56"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
+      <c r="A16" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rutinario</t>
+        </is>
+      </c>
+      <c r="B16" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descarga de la pieza terminada</t>
+        </is>
+      </c>
+      <c r="C16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El operador retira la pieza terminada de la fixtura y la coloca en el contenedor de salida</t>
+        </is>
+      </c>
+      <c r="D16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ergonomía</t>
+        </is>
+      </c>
+      <c r="E16" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Movimientos repetitivos</t>
+        </is>
+      </c>
+      <c r="F16" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fatiga muscular</t>
+        </is>
+      </c>
+      <c r="G16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Influencia</t>
+        </is>
+      </c>
+      <c r="H16" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="I16" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="J16" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K16" s="107"/>
-      <c r="L16" s="58"/>
-      <c r="M16" s="58"/>
-      <c r="N16" s="57"/>
-      <c r="O16" s="49"/>
+      <c r="K16" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ergonomía</t>
+        </is>
+      </c>
+      <c r="L16" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
+        </is>
+      </c>
+      <c r="M16" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N16" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O16" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
       <c r="P16" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7317,24 +7436,87 @@
       <c r="S16" s="57"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A17" s="55"/>
-      <c r="B17" s="55"/>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
+      <c r="A17" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rutinario</t>
+        </is>
+      </c>
+      <c r="B17" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Islas de conexión eléctrica (alimentación y sensores)</t>
+        </is>
+      </c>
+      <c r="C17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Las islas/bloques de conexión eléctrica de alimentación y de sensores quedan accesibles en el área de trabajo durante la operación normal</t>
+        </is>
+      </c>
+      <c r="D17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eléctrico</t>
+        </is>
+      </c>
+      <c r="E17" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conductores energizados</t>
+        </is>
+      </c>
+      <c r="F17" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrocución</t>
+        </is>
+      </c>
+      <c r="G17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H17" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="I17" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J17" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K17" s="107"/>
-      <c r="L17" s="58"/>
-      <c r="M17" s="58"/>
-      <c r="N17" s="57"/>
-      <c r="O17" s="49"/>
+      <c r="K17" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">detección de voltaje</t>
+        </is>
+      </c>
+      <c r="L17" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7. Adicional para intervención eléctrica: guantes dieléctricos (clase según voltaje) y calzado aislante.</t>
+        </is>
+      </c>
+      <c r="M17" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N17" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O17" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P17" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7347,24 +7529,87 @@
       <c r="S17" s="57"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A18" s="55"/>
-      <c r="B18" s="55"/>
-      <c r="C18" s="56"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="49"/>
-      <c r="G18" s="56"/>
-      <c r="H18" s="57"/>
-      <c r="I18" s="57"/>
+      <c r="A18" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B18" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arranque de la estación al inicio de turno</t>
+        </is>
+      </c>
+      <c r="C18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso 1 de 2: energiza el switch general y coloca el switch de llave en modo Automático</t>
+        </is>
+      </c>
+      <c r="D18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eléctrico</t>
+        </is>
+      </c>
+      <c r="E18" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conductores energizados</t>
+        </is>
+      </c>
+      <c r="F18" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrocución</t>
+        </is>
+      </c>
+      <c r="G18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H18" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="I18" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J18" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K18" s="107"/>
-      <c r="L18" s="58"/>
-      <c r="M18" s="58"/>
-      <c r="N18" s="57"/>
-      <c r="O18" s="49"/>
+      <c r="K18" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOTO</t>
+        </is>
+      </c>
+      <c r="L18" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7. Adicional para intervención eléctrica: guantes dieléctricos (clase según voltaje) y calzado aislante.</t>
+        </is>
+      </c>
+      <c r="M18" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N18" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O18" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P18" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7377,24 +7622,87 @@
       <c r="S18" s="57"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A19" s="55"/>
-      <c r="B19" s="55"/>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="57"/>
-      <c r="I19" s="57"/>
+      <c r="A19" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B19" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arranque de la estación al inicio de turno</t>
+        </is>
+      </c>
+      <c r="C19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso 2 de 2: inicializa el gantry (homing) y verifica que las cortinas de seguridad y el botón de reset funcionen correctamente antes de operar</t>
+        </is>
+      </c>
+      <c r="D19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecanico</t>
+        </is>
+      </c>
+      <c r="E19" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partes móviles</t>
+        </is>
+      </c>
+      <c r="F19" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atrapamiento</t>
+        </is>
+      </c>
+      <c r="G19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H19" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="I19" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J19" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K19" s="107"/>
-      <c r="L19" s="58"/>
-      <c r="M19" s="58"/>
-      <c r="N19" s="57"/>
-      <c r="O19" s="49"/>
+      <c r="K19" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sensores</t>
+        </is>
+      </c>
+      <c r="L19" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
+        </is>
+      </c>
+      <c r="M19" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N19" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O19" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P19" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7407,24 +7715,87 @@
       <c r="S19" s="57"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A20" s="55"/>
-      <c r="B20" s="55"/>
-      <c r="C20" s="56"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="56"/>
-      <c r="H20" s="57"/>
-      <c r="I20" s="57"/>
+      <c r="A20" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emergencia </t>
+        </is>
+      </c>
+      <c r="B20" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Activación del botón de paro de emergencia ante una condición insegura</t>
+        </is>
+      </c>
+      <c r="C20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El operador presiona el botón de paro de emergencia al detectar una condición insegura (atasco de pieza, invasión del área central, ruido anormal) y notifica a su supervisor/mantenimiento</t>
+        </is>
+      </c>
+      <c r="D20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecanico</t>
+        </is>
+      </c>
+      <c r="E20" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partes móviles</t>
+        </is>
+      </c>
+      <c r="F20" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atrapamiento</t>
+        </is>
+      </c>
+      <c r="G20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H20" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I20" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J20" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K20" s="107"/>
-      <c r="L20" s="58"/>
-      <c r="M20" s="58"/>
-      <c r="N20" s="57"/>
-      <c r="O20" s="49"/>
+      <c r="K20" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sensores</t>
+        </is>
+      </c>
+      <c r="L20" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
+        </is>
+      </c>
+      <c r="M20" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N20" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O20" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P20" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7437,24 +7808,87 @@
       <c r="S20" s="57"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A21" s="55"/>
-      <c r="B21" s="55"/>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="57"/>
-      <c r="I21" s="57"/>
+      <c r="A21" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emergencia </t>
+        </is>
+      </c>
+      <c r="B21" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinicio del equipo después de un paro de emergencia</t>
+        </is>
+      </c>
+      <c r="C21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Personal autorizado identifica y corrige la causa del paro (ej. libera el atasco con el switch en modo mantenimiento), verifica que el área esté despejada antes de presionar reset y reiniciar el ciclo</t>
+        </is>
+      </c>
+      <c r="D21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecanico</t>
+        </is>
+      </c>
+      <c r="E21" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partes móviles</t>
+        </is>
+      </c>
+      <c r="F21" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atrapamiento</t>
+        </is>
+      </c>
+      <c r="G21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H21" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="I21" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J21" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K21" s="107"/>
-      <c r="L21" s="58"/>
-      <c r="M21" s="58"/>
-      <c r="N21" s="57"/>
-      <c r="O21" s="49"/>
+      <c r="K21" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOTO</t>
+        </is>
+      </c>
+      <c r="L21" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
+        </is>
+      </c>
+      <c r="M21" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N21" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O21" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P21" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7467,24 +7901,87 @@
       <c r="S21" s="57"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A22" s="55"/>
-      <c r="B22" s="55"/>
-      <c r="C22" s="56"/>
-      <c r="D22" s="56"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="56"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="57"/>
+      <c r="A22" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B22" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenimiento mecánico - cambio de motor, eje o cable</t>
+        </is>
+      </c>
+      <c r="C22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso 1 de 3: cambia el switch de llave a modo Mantenimiento y bloquea/etiqueta el switch general de energía (LOTO) antes de intervenir</t>
+        </is>
+      </c>
+      <c r="D22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecanico</t>
+        </is>
+      </c>
+      <c r="E22" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partes móviles</t>
+        </is>
+      </c>
+      <c r="F22" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atrapamiento</t>
+        </is>
+      </c>
+      <c r="G22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H22" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="I22" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
       <c r="J22" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K22" s="107"/>
-      <c r="L22" s="58"/>
-      <c r="M22" s="58"/>
-      <c r="N22" s="57"/>
-      <c r="O22" s="49"/>
+      <c r="K22" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOTO</t>
+        </is>
+      </c>
+      <c r="L22" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7. Adicional para intervención eléctrica: guantes dieléctricos (clase según voltaje) y calzado aislante.</t>
+        </is>
+      </c>
+      <c r="M22" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N22" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O22" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P22" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7497,24 +7994,87 @@
       <c r="S22" s="57"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A23" s="55"/>
-      <c r="B23" s="55"/>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
+      <c r="A23" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B23" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenimiento mecánico - cambio de motor, eje o cable</t>
+        </is>
+      </c>
+      <c r="C23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso 2 de 3: reemplaza el componente (motor, eje o cable) del gantry/slider/cabezal de torque</t>
+        </is>
+      </c>
+      <c r="D23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecanico</t>
+        </is>
+      </c>
+      <c r="E23" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partes móviles</t>
+        </is>
+      </c>
+      <c r="F23" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atrapamiento</t>
+        </is>
+      </c>
+      <c r="G23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H23" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="I23" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J23" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K23" s="107"/>
-      <c r="L23" s="58"/>
-      <c r="M23" s="58"/>
-      <c r="N23" s="57"/>
-      <c r="O23" s="49"/>
+      <c r="K23" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOTO</t>
+        </is>
+      </c>
+      <c r="L23" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
+        </is>
+      </c>
+      <c r="M23" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N23" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O23" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P23" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7527,24 +8087,87 @@
       <c r="S23" s="57"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A24" s="55"/>
-      <c r="B24" s="55"/>
-      <c r="C24" s="56"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="56"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="57"/>
+      <c r="A24" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B24" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenimiento mecánico - cambio de motor, eje o cable</t>
+        </is>
+      </c>
+      <c r="C24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso 3 de 3: retira el bloqueo LOTO y realiza una prueba funcional del equipo con las cortinas de seguridad activas</t>
+        </is>
+      </c>
+      <c r="D24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecanico</t>
+        </is>
+      </c>
+      <c r="E24" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partes móviles</t>
+        </is>
+      </c>
+      <c r="F24" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atrapamiento</t>
+        </is>
+      </c>
+      <c r="G24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H24" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="I24" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J24" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K24" s="107"/>
-      <c r="L24" s="58"/>
-      <c r="M24" s="58"/>
-      <c r="N24" s="57"/>
-      <c r="O24" s="49"/>
+      <c r="K24" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sensores</t>
+        </is>
+      </c>
+      <c r="L24" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
+        </is>
+      </c>
+      <c r="M24" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N24" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O24" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P24" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7557,24 +8180,87 @@
       <c r="S24" s="57"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A25" s="55"/>
-      <c r="B25" s="55"/>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="57"/>
+      <c r="A25" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenimiento correctivo eléctrico</t>
+        </is>
+      </c>
+      <c r="C25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso 1 de 2: bloquea y etiqueta (LOTO) el switch general y abre el gabinete/panel eléctrico de la estación para diagnóstico</t>
+        </is>
+      </c>
+      <c r="D25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eléctrico</t>
+        </is>
+      </c>
+      <c r="E25" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conductores energizados</t>
+        </is>
+      </c>
+      <c r="F25" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrocución</t>
+        </is>
+      </c>
+      <c r="G25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H25" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="I25" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
       <c r="J25" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K25" s="107"/>
-      <c r="L25" s="58"/>
-      <c r="M25" s="58"/>
-      <c r="N25" s="57"/>
-      <c r="O25" s="49"/>
+      <c r="K25" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOTO</t>
+        </is>
+      </c>
+      <c r="L25" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7. Adicional para intervención eléctrica: guantes dieléctricos (clase según voltaje) y calzado aislante.</t>
+        </is>
+      </c>
+      <c r="M25" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N25" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O25" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P25" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7587,24 +8273,87 @@
       <c r="S25" s="57"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A26" s="55"/>
-      <c r="B26" s="55"/>
-      <c r="C26" s="56"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="56"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
+      <c r="A26" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B26" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenimiento correctivo eléctrico</t>
+        </is>
+      </c>
+      <c r="C26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paso 2 de 2: repara o reemplaza el componente dañado, cierra el gabinete y retira el bloqueo LOTO</t>
+        </is>
+      </c>
+      <c r="D26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eléctrico</t>
+        </is>
+      </c>
+      <c r="E26" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conductores energizados</t>
+        </is>
+      </c>
+      <c r="F26" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrocución</t>
+        </is>
+      </c>
+      <c r="G26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Control</t>
+        </is>
+      </c>
+      <c r="H26" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="I26" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="J26" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K26" s="107"/>
-      <c r="L26" s="58"/>
-      <c r="M26" s="58"/>
-      <c r="N26" s="57"/>
-      <c r="O26" s="49"/>
+      <c r="K26" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOTO</t>
+        </is>
+      </c>
+      <c r="L26" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7. Adicional para intervención eléctrica: guantes dieléctricos (clase según voltaje) y calzado aislante.</t>
+        </is>
+      </c>
+      <c r="M26" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N26" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O26" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="P26" s="61">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -7617,24 +8366,87 @@
       <c r="S26" s="57"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="55"/>
-      <c r="B27" s="55"/>
-      <c r="C27" s="56"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="56"/>
-      <c r="H27" s="57"/>
-      <c r="I27" s="57"/>
+      <c r="A27" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No rutinario</t>
+        </is>
+      </c>
+      <c r="B27" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenimiento - energía neumática residual del sistema de vacío</t>
+        </is>
+      </c>
+      <c r="C27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El personal de mantenimiento interviene la línea neumática de la electroválvula de vacío; actualmente no existe válvula de despresurización/bloqueo LOTO neumático dedicada (riesgo bajo: solo succión de baja presión, sin pistones)</t>
+        </is>
+      </c>
+      <c r="D27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecanico</t>
+        </is>
+      </c>
+      <c r="E27" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema de presión</t>
+        </is>
+      </c>
+      <c r="F27" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laceraciones</t>
+        </is>
+      </c>
+      <c r="G27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Influencia</t>
+        </is>
+      </c>
+      <c r="H27" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I27" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
       <c r="J27" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K27" s="107"/>
-      <c r="L27" s="58"/>
-      <c r="M27" s="58"/>
-      <c r="N27" s="57"/>
-      <c r="O27" s="49"/>
+      <c r="K27" s="107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspecciones periódicas</t>
+        </is>
+      </c>
+      <c r="L27" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bata/gorro de cuarto limpio (cleanroom), guantes de nitrilo, lentes de seguridad y calzado antiestático (ESD), conforme al ingreso a Cuarto Limpio ISO 7.</t>
+        </is>
+      </c>
+      <c r="M27" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16-AT40-3318-00013
+16-AT40-3318-00014
+16-AT40-3318-00015
+16-AT40-3318-00016
+16-AT40-3318-00017
+16-AT40-3318-00018
+16-AT40-3318-00019
+16-AT40-3318-00020</t>
+        </is>
+      </c>
+      <c r="N27" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EHS / Automation</t>
+        </is>
+      </c>
+      <c r="O27" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
       <c r="P27" s="61">
         <f t="shared" si="4"/>
         <v>0</v>

</xml_diff>